<commit_message>
Update preprepared scenario files to correct params and descriptions
</commit_message>
<xml_diff>
--- a/scenarios/24 hour CC running.xlsx
+++ b/scenarios/24 hour CC running.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DAAT\DAA_DES\app\inputs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DAAT\DAA_DES\scenarios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{364CD4EB-18AA-4021-91F5-A4353559ABAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41ECF070-4B7D-4057-B9E1-E20DB6815091}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{35F98327-5BE5-4FDA-9FE3-E1B3E020A414}"/>
+    <workbookView xWindow="-23148" yWindow="1632" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{35F98327-5BE5-4FDA-9FE3-E1B3E020A414}"/>
   </bookViews>
   <sheets>
     <sheet name="scenario_details" sheetId="11" r:id="rId1"/>
@@ -294,13 +294,13 @@
     <t>scenario_notes</t>
   </si>
   <si>
-    <t>Default parameters</t>
-  </si>
-  <si>
-    <t xml:space="preserve">This is a sample parameter file with some regular parameters in. </t>
-  </si>
-  <si>
     <t xml:space="preserve">There are no additional notes on this file. </t>
+  </si>
+  <si>
+    <t>24/7 helicopter coverage - critical care round the clock</t>
+  </si>
+  <si>
+    <t>This scenario sets one helicopter (H70) and its backup car (CC70) to be available 24/7/365. H70/CC70 are also set to be crewed by a critical care team at all times.</t>
   </si>
 </sst>
 </file>
@@ -426,95 +426,15 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="31">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFA400"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color theme="1"/>
-        </right>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-0.14999847407452621"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color theme="1"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color theme="1"/>
-        </top>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color theme="1"/>
-        </bottom>
-      </border>
-    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -759,6 +679,86 @@
       </fill>
       <protection locked="0" hidden="0"/>
     </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFA400"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color theme="1"/>
+        </right>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-0.14999847407452621"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="1"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color theme="1"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="1"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -778,11 +778,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{A2150AC5-74CE-48A9-BFCB-F4F61346B053}" name="Table9" displayName="Table9" ref="A1:B4" totalsRowShown="0" tableBorderDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{A2150AC5-74CE-48A9-BFCB-F4F61346B053}" name="Table9" displayName="Table9" ref="A1:B4" totalsRowShown="0" tableBorderDxfId="30">
   <autoFilter ref="A1:B4" xr:uid="{A2150AC5-74CE-48A9-BFCB-F4F61346B053}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{F0856424-C6DC-412D-B25C-8F026F7CD6E9}" name="what" dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{19C3F318-470B-475E-BB81-6C6E44750B93}" name="value" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{F0856424-C6DC-412D-B25C-8F026F7CD6E9}" name="what" dataDxfId="29"/>
+    <tableColumn id="2" xr3:uid="{19C3F318-470B-475E-BB81-6C6E44750B93}" name="value" dataDxfId="28"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -801,35 +801,35 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{6BA1A063-41E7-4CB5-905A-26CF430593FD}" name="Table2" displayName="Table2" ref="A1:E21" totalsRowShown="0" dataDxfId="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{6BA1A063-41E7-4CB5-905A-26CF430593FD}" name="Table2" displayName="Table2" ref="A1:E21" totalsRowShown="0" dataDxfId="27">
   <autoFilter ref="A1:E21" xr:uid="{6BA1A063-41E7-4CB5-905A-26CF430593FD}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{7D94D35B-078E-4674-B1CE-5BDADB0E40F1}" name="registration" dataDxfId="29"/>
-    <tableColumn id="2" xr3:uid="{87F85CD4-4878-4408-8F8D-C0C8BFCBB598}" name="callsign" dataDxfId="28"/>
-    <tableColumn id="3" xr3:uid="{BC63D893-06A9-4498-9E58-C77171B5E712}" name="model" dataDxfId="27"/>
-    <tableColumn id="4" xr3:uid="{8B732E60-F9A5-4A58-B09A-8856C6DCB309}" name="vehicle_type" dataDxfId="26"/>
-    <tableColumn id="5" xr3:uid="{66CD1ACD-7F6F-4500-B475-D2D6F6ED2307}" name="callsign_group" dataDxfId="25"/>
+    <tableColumn id="1" xr3:uid="{7D94D35B-078E-4674-B1CE-5BDADB0E40F1}" name="registration" dataDxfId="26"/>
+    <tableColumn id="2" xr3:uid="{87F85CD4-4878-4408-8F8D-C0C8BFCBB598}" name="callsign" dataDxfId="25"/>
+    <tableColumn id="3" xr3:uid="{BC63D893-06A9-4498-9E58-C77171B5E712}" name="model" dataDxfId="24"/>
+    <tableColumn id="4" xr3:uid="{8B732E60-F9A5-4A58-B09A-8856C6DCB309}" name="vehicle_type" dataDxfId="23"/>
+    <tableColumn id="5" xr3:uid="{66CD1ACD-7F6F-4500-B475-D2D6F6ED2307}" name="callsign_group" dataDxfId="22"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2FF0AB03-56FE-475B-B1B1-910C83EEE421}" name="Table3" displayName="Table3" ref="A1:H21" totalsRowShown="0" dataDxfId="24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2FF0AB03-56FE-475B-B1B1-910C83EEE421}" name="Table3" displayName="Table3" ref="A1:H21" totalsRowShown="0" dataDxfId="21">
   <autoFilter ref="A1:H21" xr:uid="{2FF0AB03-56FE-475B-B1B1-910C83EEE421}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{C8DBEC8B-3046-4DBD-B016-A8E422ADAEE6}" name="callsign" dataDxfId="23"/>
-    <tableColumn id="2" xr3:uid="{D5A51554-25D9-42A4-82A7-1DC20B1D5C7F}" name="category" dataDxfId="22"/>
-    <tableColumn id="3" xr3:uid="{083D7748-F407-4874-AEE3-F57C80BB60CB}" name="vehicle_type" dataDxfId="21">
+    <tableColumn id="1" xr3:uid="{C8DBEC8B-3046-4DBD-B016-A8E422ADAEE6}" name="callsign" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{D5A51554-25D9-42A4-82A7-1DC20B1D5C7F}" name="category" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{083D7748-F407-4874-AEE3-F57C80BB60CB}" name="vehicle_type" dataDxfId="18">
       <calculatedColumnFormula>IF(ISBLANK(Table3[[#This Row],[callsign]]), "", VLOOKUP(Table3[[#This Row],[callsign]],Table2[[#All],[callsign]:[vehicle_type]],3,FALSE))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{F8436158-780C-4799-95D0-FA534C9C1BBA}" name="callsign_group" dataDxfId="20">
+    <tableColumn id="4" xr3:uid="{F8436158-780C-4799-95D0-FA534C9C1BBA}" name="callsign_group" dataDxfId="17">
       <calculatedColumnFormula>IF(ISBLANK(Table3[[#This Row],[callsign]]),"",VLOOKUP(Table3[[#This Row],[callsign]],Table2[[callsign]:[callsign_group]],4,FALSE))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{748FACE2-04C4-49AA-860C-6DC2CA8F9616}" name="summer_start" dataDxfId="19"/>
-    <tableColumn id="6" xr3:uid="{57A2D311-6390-401A-9AC0-6CD26AC91087}" name="winter_start" dataDxfId="18"/>
-    <tableColumn id="7" xr3:uid="{0C1D6883-A527-469B-906E-ACE4ADBD99BC}" name="summer_end" dataDxfId="17"/>
-    <tableColumn id="8" xr3:uid="{CB8009A1-EE5E-4E82-AE4B-A7BB0D34F6B0}" name="winter_end" dataDxfId="16"/>
+    <tableColumn id="5" xr3:uid="{748FACE2-04C4-49AA-860C-6DC2CA8F9616}" name="summer_start" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{57A2D311-6390-401A-9AC0-6CD26AC91087}" name="winter_start" dataDxfId="15"/>
+    <tableColumn id="7" xr3:uid="{0C1D6883-A527-469B-906E-ACE4ADBD99BC}" name="summer_end" dataDxfId="14"/>
+    <tableColumn id="8" xr3:uid="{CB8009A1-EE5E-4E82-AE4B-A7BB0D34F6B0}" name="winter_end" dataDxfId="13"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -839,11 +839,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{F3C351CF-682F-4BF7-B3CD-24B10E4A2F0D}" name="Table8" displayName="Table8" ref="B1:D19" totalsRowShown="0">
   <autoFilter ref="B1:D19" xr:uid="{F3C351CF-682F-4BF7-B3CD-24B10E4A2F0D}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{910E7A2A-0672-402C-B39B-5F4EFFE22D82}" name="vehicle_type" dataDxfId="15">
+    <tableColumn id="1" xr3:uid="{910E7A2A-0672-402C-B39B-5F4EFFE22D82}" name="vehicle_type" dataDxfId="12">
       <calculatedColumnFormula>IF(ISBLANK(A2),"", VLOOKUP(A2,callsign_registration_lookup!C1:E6,2,FALSE))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{D8B7BF02-3B19-4DC4-B9A4-EDEC06128AD9}" name="service_schedule_months" dataDxfId="14"/>
-    <tableColumn id="3" xr3:uid="{52C2F997-5183-4694-B686-C7FFF875B647}" name="service_duration_weeks" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{D8B7BF02-3B19-4DC4-B9A4-EDEC06128AD9}" name="service_schedule_months" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{52C2F997-5183-4694-B686-C7FFF875B647}" name="service_duration_weeks" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -864,19 +864,19 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{B52178EC-48A3-4EAB-A281-FC4D4E29EBFD}" name="Table11" displayName="Table11" ref="A1:C7" totalsRowShown="0">
   <autoFilter ref="A1:C7" xr:uid="{B52178EC-48A3-4EAB-A281-FC4D4E29EBFD}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{309A14F6-9A64-48F1-9FAE-814E60D5F781}" name="time" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{EB9F8E5F-5B1B-4C3B-B477-7D6B1C11C11F}" name="min_value_mins" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{AA844072-6D2B-4C5F-AAB4-2FA58A23BD97}" name="max_value_mins" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{309A14F6-9A64-48F1-9FAE-814E60D5F781}" name="time" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{EB9F8E5F-5B1B-4C3B-B477-7D6B1C11C11F}" name="min_value_mins" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{AA844072-6D2B-4C5F-AAB4-2FA58A23BD97}" name="max_value_mins" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{447F2987-19D0-4529-9F11-F3A4C3B081CC}" name="Table10" displayName="Table10" ref="B1:B20" totalsRowShown="0" dataDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{447F2987-19D0-4529-9F11-F3A4C3B081CC}" name="Table10" displayName="Table10" ref="B1:B20" totalsRowShown="0" dataDxfId="6">
   <autoFilter ref="B1:B20" xr:uid="{447F2987-19D0-4529-9F11-F3A4C3B081CC}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{3F69728E-661E-4266-B4A5-B5ECD8439827}" name="last_service" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{3F69728E-661E-4266-B4A5-B5ECD8439827}" name="last_service" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -886,11 +886,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{42097D3F-3BEA-464C-9C83-98399518AAC6}" name="Table5" displayName="Table5" ref="A1:C71" totalsRowShown="0">
   <autoFilter ref="A1:C71" xr:uid="{42097D3F-3BEA-464C-9C83-98399518AAC6}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{B8A9B6B6-A29A-43D5-8097-C40C62115672}" name="year" dataDxfId="7">
+    <tableColumn id="1" xr3:uid="{B8A9B6B6-A29A-43D5-8097-C40C62115672}" name="year" dataDxfId="4">
       <calculatedColumnFormula>IF(ISBLANK(B2), "", YEAR(B2))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{5CC3236A-0549-4C18-B5F2-35A3935BCD55}" name="start_date" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{20E5EE56-B6F2-4D76-82F2-881E011DF77B}" name="end_date" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{5CC3236A-0549-4C18-B5F2-35A3935BCD55}" name="start_date" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{20E5EE56-B6F2-4D76-82F2-881E011DF77B}" name="end_date" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -900,8 +900,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E2677EC5-725F-4393-AF15-F56183802269}" name="Table1" displayName="Table1" ref="A1:B8" totalsRowShown="0">
   <autoFilter ref="A1:B8" xr:uid="{E2677EC5-725F-4393-AF15-F56183802269}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{99B5D3F1-FB03-439A-8D7C-566528BE4775}" name="parameter" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{BC693C23-ACAE-4C24-89FD-3BA288AA600E}" name="value" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{99B5D3F1-FB03-439A-8D7C-566528BE4775}" name="parameter" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{BC693C23-ACAE-4C24-89FD-3BA288AA600E}" name="value" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1225,13 +1225,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9543A6F1-AEF6-457F-88F4-18CC0389619D}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="88.109375" customWidth="1"/>
+    <col min="2" max="2" width="88.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>27</v>
       </c>
@@ -1239,28 +1239,28 @@
         <v>62</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>72</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="214.8" customHeight="1" x14ac:dyDescent="0.3">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="214.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>73</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="118.8" customHeight="1" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="118.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>74</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -1275,14 +1275,14 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1B29D2C-108A-4FF4-8D5D-63ADEC51A17D}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.33203125" customWidth="1"/>
-    <col min="3" max="3" width="18.88671875" customWidth="1"/>
+    <col min="1" max="1" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.28515625" customWidth="1"/>
+    <col min="3" max="3" width="18.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>58</v>
       </c>
@@ -1293,7 +1293,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>23</v>
       </c>
@@ -1304,7 +1304,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>25</v>
       </c>
@@ -1315,52 +1315,52 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>56</v>
       </c>
@@ -1376,16 +1376,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16EE6093-5A5B-497D-B656-3B9060F09677}">
   <dimension ref="A1:E21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="20.88671875" customWidth="1"/>
-    <col min="3" max="3" width="30.33203125" customWidth="1"/>
-    <col min="4" max="4" width="15.109375" customWidth="1"/>
-    <col min="5" max="5" width="17.5546875" customWidth="1"/>
+    <col min="2" max="2" width="20.85546875" customWidth="1"/>
+    <col min="3" max="3" width="30.28515625" customWidth="1"/>
+    <col min="4" max="4" width="15.140625" customWidth="1"/>
+    <col min="5" max="5" width="17.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1402,7 +1402,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>3</v>
       </c>
@@ -1419,7 +1419,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>6</v>
       </c>
@@ -1436,7 +1436,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>9</v>
       </c>
@@ -1453,7 +1453,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>10</v>
       </c>
@@ -1470,7 +1470,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>11</v>
       </c>
@@ -1487,105 +1487,105 @@
         <v>72</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="7"/>
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
       <c r="E7" s="7"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="7"/>
       <c r="B8" s="7"/>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
       <c r="E8" s="7"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
       <c r="E9" s="7"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="7"/>
       <c r="B10" s="7"/>
       <c r="C10" s="7"/>
       <c r="D10" s="7"/>
       <c r="E10" s="7"/>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="7"/>
       <c r="B11" s="7"/>
       <c r="C11" s="7"/>
       <c r="D11" s="7"/>
       <c r="E11" s="7"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="7"/>
       <c r="B12" s="7"/>
       <c r="C12" s="7"/>
       <c r="D12" s="7"/>
       <c r="E12" s="7"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="7"/>
       <c r="B13" s="7"/>
       <c r="C13" s="7"/>
       <c r="D13" s="7"/>
       <c r="E13" s="7"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="7"/>
       <c r="B14" s="7"/>
       <c r="C14" s="7"/>
       <c r="D14" s="7"/>
       <c r="E14" s="7"/>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="7"/>
       <c r="B15" s="7"/>
       <c r="C15" s="7"/>
       <c r="D15" s="7"/>
       <c r="E15" s="7"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="7"/>
       <c r="B16" s="7"/>
       <c r="C16" s="7"/>
       <c r="D16" s="7"/>
       <c r="E16" s="7"/>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="7"/>
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
       <c r="D17" s="7"/>
       <c r="E17" s="7"/>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="7"/>
       <c r="B18" s="7"/>
       <c r="C18" s="7"/>
       <c r="D18" s="7"/>
       <c r="E18" s="7"/>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="7"/>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
       <c r="D19" s="7"/>
       <c r="E19" s="7"/>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="7"/>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
       <c r="D20" s="7"/>
       <c r="E20" s="7"/>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="7"/>
       <c r="B21" s="7"/>
       <c r="C21" s="7"/>
@@ -1616,19 +1616,19 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3E65222-ED7F-4312-B1BC-43F34F9AFBA9}">
   <dimension ref="A1:H21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.109375" customWidth="1"/>
-    <col min="2" max="2" width="15.5546875" customWidth="1"/>
+    <col min="1" max="1" width="17.140625" customWidth="1"/>
+    <col min="2" max="2" width="15.5703125" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="19.109375" customWidth="1"/>
-    <col min="5" max="5" width="18.6640625" customWidth="1"/>
-    <col min="6" max="6" width="17.6640625" customWidth="1"/>
-    <col min="7" max="7" width="18.109375" customWidth="1"/>
+    <col min="4" max="4" width="19.140625" customWidth="1"/>
+    <col min="5" max="5" width="18.7109375" customWidth="1"/>
+    <col min="6" max="6" width="17.7109375" customWidth="1"/>
+    <col min="7" max="7" width="18.140625" customWidth="1"/>
     <col min="8" max="8" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -1654,7 +1654,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>4</v>
       </c>
@@ -1682,12 +1682,12 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C3" s="1" t="str">
         <f>IF(ISBLANK(Table3[[#This Row],[callsign]]), "", VLOOKUP(Table3[[#This Row],[callsign]],Table2[[#All],[callsign]:[vehicle_type]],3,FALSE))</f>
@@ -1704,13 +1704,13 @@
         <v>19</v>
       </c>
       <c r="G3" s="7">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="H3" s="7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>12</v>
       </c>
@@ -1738,12 +1738,12 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>12</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C5" s="1" t="str">
         <f>IF(ISBLANK(Table3[[#This Row],[callsign]]), "", VLOOKUP(Table3[[#This Row],[callsign]],Table2[[#All],[callsign]:[vehicle_type]],3,FALSE))</f>
@@ -1760,13 +1760,13 @@
         <v>19</v>
       </c>
       <c r="G5" s="7">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="H5" s="7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>7</v>
       </c>
@@ -1794,7 +1794,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>13</v>
       </c>
@@ -1822,7 +1822,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>14</v>
       </c>
@@ -1850,7 +1850,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="1" t="str">
@@ -1866,7 +1866,7 @@
       <c r="G9" s="7"/>
       <c r="H9" s="7"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="7"/>
       <c r="B10" s="7"/>
       <c r="C10" s="1" t="str">
@@ -1882,7 +1882,7 @@
       <c r="G10" s="7"/>
       <c r="H10" s="7"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="7"/>
       <c r="B11" s="7"/>
       <c r="C11" s="1" t="str">
@@ -1898,7 +1898,7 @@
       <c r="G11" s="7"/>
       <c r="H11" s="7"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="7"/>
       <c r="B12" s="7"/>
       <c r="C12" s="1" t="str">
@@ -1914,7 +1914,7 @@
       <c r="G12" s="7"/>
       <c r="H12" s="7"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="7"/>
       <c r="B13" s="7"/>
       <c r="C13" s="1" t="str">
@@ -1930,7 +1930,7 @@
       <c r="G13" s="7"/>
       <c r="H13" s="7"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="7"/>
       <c r="B14" s="7"/>
       <c r="C14" s="1" t="str">
@@ -1946,7 +1946,7 @@
       <c r="G14" s="7"/>
       <c r="H14" s="7"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="7"/>
       <c r="B15" s="7"/>
       <c r="C15" s="1" t="str">
@@ -1962,7 +1962,7 @@
       <c r="G15" s="7"/>
       <c r="H15" s="7"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="7"/>
       <c r="B16" s="7"/>
       <c r="C16" s="1" t="str">
@@ -1978,7 +1978,7 @@
       <c r="G16" s="7"/>
       <c r="H16" s="7"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="7"/>
       <c r="B17" s="7"/>
       <c r="C17" s="1" t="str">
@@ -1994,7 +1994,7 @@
       <c r="G17" s="7"/>
       <c r="H17" s="7"/>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="7"/>
       <c r="B18" s="7"/>
       <c r="C18" s="1" t="str">
@@ -2010,7 +2010,7 @@
       <c r="G18" s="7"/>
       <c r="H18" s="7"/>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="7"/>
       <c r="B19" s="7"/>
       <c r="C19" s="1" t="str">
@@ -2026,7 +2026,7 @@
       <c r="G19" s="7"/>
       <c r="H19" s="7"/>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="7"/>
       <c r="B20" s="7"/>
       <c r="C20" s="1" t="str">
@@ -2042,7 +2042,7 @@
       <c r="G20" s="7"/>
       <c r="H20" s="7"/>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="7"/>
       <c r="B21" s="7"/>
       <c r="C21" s="1" t="str">
@@ -2082,15 +2082,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4472C9B-3E4C-4DDF-8989-3DE050C2A20C}">
   <dimension ref="A1:D19"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.109375" customWidth="1"/>
-    <col min="3" max="3" width="27.109375" customWidth="1"/>
-    <col min="4" max="4" width="25.5546875" customWidth="1"/>
+    <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.140625" customWidth="1"/>
+    <col min="3" max="3" width="27.140625" customWidth="1"/>
+    <col min="4" max="4" width="25.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>2</v>
       </c>
@@ -2104,7 +2104,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="str" cm="1">
         <f t="array" ref="A2:A4">_xlfn.UNIQUE(_xlfn._xlws.FILTER(Table2[model], Table2[model] &lt;&gt; ""))</f>
         <v>Airbus H145</v>
@@ -2120,7 +2120,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="str">
         <v>Airbus EC135</v>
       </c>
@@ -2135,7 +2135,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="str">
         <v>Volvo XC90</v>
       </c>
@@ -2150,7 +2150,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="4" t="str">
         <f>IF(ISBLANK(A5),"", VLOOKUP(A5,callsign_registration_lookup!C4:E9,2,FALSE))</f>
@@ -2159,7 +2159,7 @@
       <c r="C5" s="8"/>
       <c r="D5" s="8"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
       <c r="B6" s="4" t="str">
         <f>IF(ISBLANK(A6),"", VLOOKUP(A6,callsign_registration_lookup!C5:E10,2,FALSE))</f>
@@ -2168,7 +2168,7 @@
       <c r="C6" s="8"/>
       <c r="D6" s="8"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="3"/>
       <c r="B7" s="4" t="str">
         <f>IF(ISBLANK(A7),"", VLOOKUP(A7,callsign_registration_lookup!C6:E11,2,FALSE))</f>
@@ -2177,7 +2177,7 @@
       <c r="C7" s="8"/>
       <c r="D7" s="8"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="3"/>
       <c r="B8" s="4" t="str">
         <f>IF(ISBLANK(A8),"", VLOOKUP(A8,callsign_registration_lookup!C7:E12,2,FALSE))</f>
@@ -2186,7 +2186,7 @@
       <c r="C8" s="8"/>
       <c r="D8" s="8"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
       <c r="B9" s="4" t="str">
         <f>IF(ISBLANK(A9),"", VLOOKUP(A9,callsign_registration_lookup!C8:E13,2,FALSE))</f>
@@ -2195,7 +2195,7 @@
       <c r="C9" s="8"/>
       <c r="D9" s="8"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="3"/>
       <c r="B10" s="4" t="str">
         <f>IF(ISBLANK(A10),"", VLOOKUP(A10,callsign_registration_lookup!C9:E14,2,FALSE))</f>
@@ -2204,7 +2204,7 @@
       <c r="C10" s="8"/>
       <c r="D10" s="8"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="3"/>
       <c r="B11" s="4" t="str">
         <f>IF(ISBLANK(A11),"", VLOOKUP(A11,callsign_registration_lookup!C10:E15,2,FALSE))</f>
@@ -2213,7 +2213,7 @@
       <c r="C11" s="8"/>
       <c r="D11" s="8"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
       <c r="B12" s="4" t="str">
         <f>IF(ISBLANK(A12),"", VLOOKUP(A12,callsign_registration_lookup!C11:E16,2,FALSE))</f>
@@ -2222,7 +2222,7 @@
       <c r="C12" s="8"/>
       <c r="D12" s="8"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="3"/>
       <c r="B13" s="4" t="str">
         <f>IF(ISBLANK(A13),"", VLOOKUP(A13,callsign_registration_lookup!C12:E17,2,FALSE))</f>
@@ -2231,7 +2231,7 @@
       <c r="C13" s="8"/>
       <c r="D13" s="8"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>
       <c r="B14" s="4" t="str">
         <f>IF(ISBLANK(A14),"", VLOOKUP(A14,callsign_registration_lookup!C13:E18,2,FALSE))</f>
@@ -2240,7 +2240,7 @@
       <c r="C14" s="8"/>
       <c r="D14" s="8"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
       <c r="B15" s="4" t="str">
         <f>IF(ISBLANK(A15),"", VLOOKUP(A15,callsign_registration_lookup!C14:E19,2,FALSE))</f>
@@ -2249,7 +2249,7 @@
       <c r="C15" s="8"/>
       <c r="D15" s="8"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
       <c r="B16" s="4" t="str">
         <f>IF(ISBLANK(A16),"", VLOOKUP(A16,callsign_registration_lookup!C15:E20,2,FALSE))</f>
@@ -2258,7 +2258,7 @@
       <c r="C16" s="8"/>
       <c r="D16" s="8"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="3"/>
       <c r="B17" s="4" t="str">
         <f>IF(ISBLANK(A17),"", VLOOKUP(A17,callsign_registration_lookup!C16:E21,2,FALSE))</f>
@@ -2267,7 +2267,7 @@
       <c r="C17" s="8"/>
       <c r="D17" s="8"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="3"/>
       <c r="B18" s="4" t="str">
         <f>IF(ISBLANK(A18),"", VLOOKUP(A18,callsign_registration_lookup!C17:E22,2,FALSE))</f>
@@ -2276,7 +2276,7 @@
       <c r="C18" s="8"/>
       <c r="D18" s="8"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="3"/>
       <c r="B19" s="4" t="str">
         <f>IF(ISBLANK(A19),"", VLOOKUP(A19,callsign_registration_lookup!C18:E23,2,FALSE))</f>
@@ -2297,12 +2297,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF8280D3-5117-4A4B-955E-D11A20FA9E1E}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>27</v>
       </c>
@@ -2310,7 +2310,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>31</v>
       </c>
@@ -2318,7 +2318,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>33</v>
       </c>
@@ -2326,7 +2326,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>29</v>
       </c>
@@ -2335,7 +2335,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>30</v>
       </c>
@@ -2356,14 +2356,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FD2B715-A401-4418-8566-F4AD33A9A218}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.5546875" customWidth="1"/>
-    <col min="3" max="3" width="20.6640625" customWidth="1"/>
+    <col min="1" max="1" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.5703125" customWidth="1"/>
+    <col min="3" max="3" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>38</v>
       </c>
@@ -2374,7 +2374,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>41</v>
       </c>
@@ -2385,7 +2385,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>42</v>
       </c>
@@ -2396,7 +2396,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>43</v>
       </c>
@@ -2407,7 +2407,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>44</v>
       </c>
@@ -2418,7 +2418,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>45</v>
       </c>
@@ -2429,7 +2429,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>46</v>
       </c>
@@ -2458,13 +2458,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC77B55E-07E5-4BCD-A568-968CBEC9848C}">
   <dimension ref="A1:B20"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.5546875" customWidth="1"/>
-    <col min="2" max="2" width="21.33203125" customWidth="1"/>
+    <col min="1" max="1" width="16.5703125" customWidth="1"/>
+    <col min="2" max="2" width="21.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -2472,7 +2472,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="str" cm="1">
         <f t="array" ref="A2:A6">_xlfn.UNIQUE(_xlfn._xlws.FILTER(Table2[registration], Table2[registration] &lt;&gt; ""))</f>
         <v>g-daas</v>
@@ -2481,7 +2481,7 @@
         <v>44565</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="str">
         <v>g-daan</v>
       </c>
@@ -2489,7 +2489,7 @@
         <v>44640</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="str">
         <v>cc70</v>
       </c>
@@ -2497,7 +2497,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="str">
         <v>cc71</v>
       </c>
@@ -2505,7 +2505,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="str">
         <v>cc72</v>
       </c>
@@ -2513,59 +2513,59 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="3"/>
       <c r="B7" s="8"/>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="3"/>
       <c r="B8" s="8"/>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
       <c r="B9" s="8"/>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="3"/>
       <c r="B10" s="8"/>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="3"/>
       <c r="B11" s="8"/>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
       <c r="B12" s="8"/>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="3"/>
       <c r="B13" s="8"/>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>
       <c r="B14" s="8"/>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
       <c r="B15" s="8"/>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
       <c r="B16" s="8"/>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="3"/>
       <c r="B17" s="8"/>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="3"/>
       <c r="B18" s="8"/>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="3"/>
       <c r="B19" s="8"/>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="3"/>
       <c r="B20" s="8"/>
     </row>
@@ -2581,13 +2581,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEFAD79A-DE70-441B-AB11-9139E7B03EF5}">
   <dimension ref="A1:C71"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="11.33203125" customWidth="1"/>
-    <col min="3" max="3" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.28515625" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>69</v>
       </c>
@@ -2598,7 +2598,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="4">
         <f t="shared" ref="A2:A43" si="0">IF(ISBLANK(B2), "", YEAR(B2))</f>
         <v>2023</v>
@@ -2610,7 +2610,7 @@
         <v>44928</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="4">
         <f t="shared" si="0"/>
         <v>2023</v>
@@ -2622,7 +2622,7 @@
         <v>44974</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
         <f t="shared" si="0"/>
         <v>2023</v>
@@ -2634,7 +2634,7 @@
         <v>45033</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="4">
         <f t="shared" si="0"/>
         <v>2023</v>
@@ -2646,7 +2646,7 @@
         <v>45081</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
         <f t="shared" si="0"/>
         <v>2023</v>
@@ -2658,7 +2658,7 @@
         <v>45173</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="4">
         <f t="shared" si="0"/>
         <v>2023</v>
@@ -2670,7 +2670,7 @@
         <v>45228</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="4">
         <f t="shared" si="0"/>
         <v>2023</v>
@@ -2682,7 +2682,7 @@
         <v>45291</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
         <f t="shared" si="0"/>
         <v>2024</v>
@@ -2694,7 +2694,7 @@
         <v>45292</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
         <f t="shared" si="0"/>
         <v>2024</v>
@@ -2706,7 +2706,7 @@
         <v>45338</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="4">
         <f t="shared" si="0"/>
         <v>2024</v>
@@ -2718,7 +2718,7 @@
         <v>45396</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="4">
         <f t="shared" si="0"/>
         <v>2024</v>
@@ -2730,7 +2730,7 @@
         <v>45445</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="4">
         <f t="shared" si="0"/>
         <v>2024</v>
@@ -2742,7 +2742,7 @@
         <v>45537</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="4">
         <f t="shared" si="0"/>
         <v>2024</v>
@@ -2754,7 +2754,7 @@
         <v>45599</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="4">
         <f t="shared" si="0"/>
         <v>2024</v>
@@ -2766,7 +2766,7 @@
         <v>45657</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="4">
         <f t="shared" si="0"/>
         <v>2025</v>
@@ -2778,7 +2778,7 @@
         <v>45662</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="4">
         <f t="shared" si="0"/>
         <v>2025</v>
@@ -2790,7 +2790,7 @@
         <v>45711</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="4">
         <f t="shared" si="0"/>
         <v>2025</v>
@@ -2802,7 +2802,7 @@
         <v>45768</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="4">
         <f t="shared" si="0"/>
         <v>2025</v>
@@ -2814,7 +2814,7 @@
         <v>45809</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="4">
         <f t="shared" si="0"/>
         <v>2025</v>
@@ -2826,7 +2826,7 @@
         <v>45901</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="4">
         <f t="shared" si="0"/>
         <v>2025</v>
@@ -2838,7 +2838,7 @@
         <v>45963</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="4">
         <f t="shared" si="0"/>
         <v>2025</v>
@@ -2850,7 +2850,7 @@
         <v>46022</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="4">
         <f t="shared" si="0"/>
         <v>2026</v>
@@ -2862,7 +2862,7 @@
         <v>46026</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="4">
         <f t="shared" si="0"/>
         <v>2026</v>
@@ -2874,7 +2874,7 @@
         <v>46075</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="4">
         <f t="shared" si="0"/>
         <v>2026</v>
@@ -2886,7 +2886,7 @@
         <v>46131</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="4">
         <f t="shared" si="0"/>
         <v>2026</v>
@@ -2898,7 +2898,7 @@
         <v>46173</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="4">
         <f t="shared" si="0"/>
         <v>2026</v>
@@ -2910,7 +2910,7 @@
         <v>46267</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="4">
         <f t="shared" si="0"/>
         <v>2026</v>
@@ -2922,7 +2922,7 @@
         <v>46296</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="4">
         <f t="shared" si="0"/>
         <v>2026</v>
@@ -2934,7 +2934,7 @@
         <v>46387</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="4">
         <f t="shared" si="0"/>
         <v>2027</v>
@@ -2946,7 +2946,7 @@
         <v>46390</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="4">
         <f t="shared" si="0"/>
         <v>2027</v>
@@ -2958,7 +2958,7 @@
         <v>46439</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="4">
         <f t="shared" si="0"/>
         <v>2027</v>
@@ -2970,7 +2970,7 @@
         <v>46488</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="4">
         <f t="shared" si="0"/>
         <v>2027</v>
@@ -2982,7 +2982,7 @@
         <v>46544</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="4">
         <f t="shared" si="0"/>
         <v>2027</v>
@@ -2994,7 +2994,7 @@
         <v>46631</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="4">
         <f t="shared" si="0"/>
         <v>2027</v>
@@ -3006,7 +3006,7 @@
         <v>46691</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="4">
         <f t="shared" si="0"/>
         <v>2027</v>
@@ -3018,7 +3018,7 @@
         <v>46752</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3026,7 +3026,7 @@
       <c r="B37" s="7"/>
       <c r="C37" s="7"/>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3034,7 +3034,7 @@
       <c r="B38" s="7"/>
       <c r="C38" s="7"/>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3042,7 +3042,7 @@
       <c r="B39" s="7"/>
       <c r="C39" s="7"/>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3050,7 +3050,7 @@
       <c r="B40" s="7"/>
       <c r="C40" s="7"/>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3058,7 +3058,7 @@
       <c r="B41" s="7"/>
       <c r="C41" s="7"/>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3066,7 +3066,7 @@
       <c r="B42" s="7"/>
       <c r="C42" s="7"/>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" s="4" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -3074,7 +3074,7 @@
       <c r="B43" s="7"/>
       <c r="C43" s="7"/>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="str">
         <f t="shared" ref="A44:A71" si="1">IF(ISBLANK(B44), "", YEAR(B44))</f>
         <v/>
@@ -3082,7 +3082,7 @@
       <c r="B44" s="7"/>
       <c r="C44" s="7"/>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3090,7 +3090,7 @@
       <c r="B45" s="7"/>
       <c r="C45" s="7"/>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3098,7 +3098,7 @@
       <c r="B46" s="7"/>
       <c r="C46" s="7"/>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3106,7 +3106,7 @@
       <c r="B47" s="7"/>
       <c r="C47" s="7"/>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3114,7 +3114,7 @@
       <c r="B48" s="7"/>
       <c r="C48" s="7"/>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3122,7 +3122,7 @@
       <c r="B49" s="7"/>
       <c r="C49" s="7"/>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3130,7 +3130,7 @@
       <c r="B50" s="7"/>
       <c r="C50" s="7"/>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3138,7 +3138,7 @@
       <c r="B51" s="7"/>
       <c r="C51" s="7"/>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3146,7 +3146,7 @@
       <c r="B52" s="7"/>
       <c r="C52" s="7"/>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3154,7 +3154,7 @@
       <c r="B53" s="7"/>
       <c r="C53" s="7"/>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3162,7 +3162,7 @@
       <c r="B54" s="7"/>
       <c r="C54" s="7"/>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3170,7 +3170,7 @@
       <c r="B55" s="7"/>
       <c r="C55" s="7"/>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3178,7 +3178,7 @@
       <c r="B56" s="7"/>
       <c r="C56" s="7"/>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3186,7 +3186,7 @@
       <c r="B57" s="7"/>
       <c r="C57" s="7"/>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3194,7 +3194,7 @@
       <c r="B58" s="7"/>
       <c r="C58" s="7"/>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3202,7 +3202,7 @@
       <c r="B59" s="7"/>
       <c r="C59" s="7"/>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3210,7 +3210,7 @@
       <c r="B60" s="7"/>
       <c r="C60" s="7"/>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3218,7 +3218,7 @@
       <c r="B61" s="7"/>
       <c r="C61" s="7"/>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3226,7 +3226,7 @@
       <c r="B62" s="7"/>
       <c r="C62" s="7"/>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3234,7 +3234,7 @@
       <c r="B63" s="7"/>
       <c r="C63" s="7"/>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3242,7 +3242,7 @@
       <c r="B64" s="7"/>
       <c r="C64" s="7"/>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3250,7 +3250,7 @@
       <c r="B65" s="7"/>
       <c r="C65" s="7"/>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3258,7 +3258,7 @@
       <c r="B66" s="7"/>
       <c r="C66" s="7"/>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3266,7 +3266,7 @@
       <c r="B67" s="7"/>
       <c r="C67" s="7"/>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3274,7 +3274,7 @@
       <c r="B68" s="7"/>
       <c r="C68" s="7"/>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3282,7 +3282,7 @@
       <c r="B69" s="7"/>
       <c r="C69" s="7"/>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3290,7 +3290,7 @@
       <c r="B70" s="7"/>
       <c r="C70" s="7"/>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" s="4" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3310,13 +3310,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B548ABE7-8EC4-45E9-9646-4F60214B4C5B}">
   <dimension ref="A1:B21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="34.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.5546875" customWidth="1"/>
+    <col min="1" max="1" width="34.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>61</v>
       </c>
@@ -3324,7 +3324,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>60</v>
       </c>
@@ -3332,7 +3332,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>63</v>
       </c>
@@ -3340,7 +3340,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>64</v>
       </c>
@@ -3348,7 +3348,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>65</v>
       </c>
@@ -3356,7 +3356,7 @@
         <v>44927</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>66</v>
       </c>
@@ -3364,7 +3364,7 @@
         <v>0.33333333333333331</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>67</v>
       </c>
@@ -3372,7 +3372,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>68</v>
       </c>
@@ -3380,43 +3380,43 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B9" s="6"/>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B10" s="6"/>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B11" s="6"/>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B12" s="6"/>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B13" s="6"/>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B14" s="6"/>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B15" s="6"/>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B16" s="6"/>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" s="6"/>
     </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" s="6"/>
     </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B19" s="6"/>
     </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B20" s="6"/>
     </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B21" s="6"/>
     </row>
   </sheetData>

</xml_diff>